<commit_message>
Refactorizar comparacion ML vs Kriging y actualizar pipeline
- 00. coords.py: guardar coords bloque matcheado (Este_val/Norte_val/Cota_val) en CSV
- 04. comparacion_ml_vs_kriging.py: reemplaza LOOCV por entrenamiento 100% + prediccion en bloque
  mas cercano. Modelos: KNN, RandomForest, GradientBoosting, XGBoost con params fijos.
  Tabla final incluye diferencia porcentual de R2 vs kriging.
- Actualizar imagenes de comparacion ML vs kriging

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/processed/Obs/metricas_ml_vs_kriging.xlsx
+++ b/data/processed/Obs/metricas_ml_vs_kriging.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,15 +436,20 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>delta_r2_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>r2</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>rmse</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>mape_pct</t>
         </is>
@@ -453,97 +458,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RandomForest</t>
+          <t>Kriging</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2373028681901077</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>5.785234481717601</v>
+        <v>0.7959994903761819</v>
       </c>
       <c r="D2" t="n">
-        <v>22.51487531354338</v>
+        <v>2.991992741789238</v>
+      </c>
+      <c r="E2" t="n">
+        <v>10.50657384520661</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GradientBoosting</t>
+          <t>KNN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.174114730449674</v>
+        <v>-20.90188829303729</v>
       </c>
       <c r="C3" t="n">
-        <v>6.020114750899377</v>
+        <v>0.6296205660846063</v>
       </c>
       <c r="D3" t="n">
-        <v>23.32601213054951</v>
+        <v>4.031515568543076</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13.33256722400612</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>GradientBoosting</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1666160778278581</v>
+        <v>-51.38855464311287</v>
       </c>
       <c r="C4" t="n">
-        <v>6.04738291072193</v>
+        <v>0.3869468573053176</v>
       </c>
       <c r="D4" t="n">
-        <v>23.38215331541188</v>
+        <v>5.186733941551842</v>
+      </c>
+      <c r="E4" t="n">
+        <v>19.55692117189602</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KNN</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1480993166537994</v>
+        <v>-54.24426129457993</v>
       </c>
       <c r="C5" t="n">
-        <v>6.114196509353249</v>
+        <v>0.3642154469130011</v>
       </c>
       <c r="D5" t="n">
-        <v>23.00305987521469</v>
+        <v>5.282018227339186</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19.98871761707565</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SVR</t>
+          <t>RandomForest</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.08454463405418033</v>
+        <v>-56.98237786328117</v>
       </c>
       <c r="C6" t="n">
-        <v>6.33816435635594</v>
+        <v>0.3424200529802335</v>
       </c>
       <c r="D6" t="n">
-        <v>25.18246143791941</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>-0.0224993396441231</v>
-      </c>
-      <c r="C7" t="n">
-        <v>6.698482507219894</v>
-      </c>
-      <c r="D7" t="n">
-        <v>26.59349546455573</v>
+        <v>5.371792022318755</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20.27325930605141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar analisis geostadistico y refactorizar comparacion ML vs Kriging
- 04.: exporta predicciones a data/results/ para uso en 05.; corrige delta R2 a diferencia absoluta en puntos porcentuales
- 05. (nuevo): histogramas normalizados y graficas de deriva espacial (Este, Norte, Cota) comparando Original, Kriging y modelos ML con paleta profesional

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/processed/Obs/metricas_ml_vs_kriging.xlsx
+++ b/data/processed/Obs/metricas_ml_vs_kriging.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-20.90188829303729</v>
+        <v>-16.63789242915756</v>
       </c>
       <c r="C3" t="n">
         <v>0.6296205660846063</v>
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-51.38855464311287</v>
+        <v>-40.90526330708643</v>
       </c>
       <c r="C4" t="n">
         <v>0.3869468573053176</v>
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-54.24426129457993</v>
+        <v>-43.17840434631808</v>
       </c>
       <c r="C5" t="n">
         <v>0.3642154469130011</v>
@@ -538,16 +538,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-56.98237786328117</v>
+        <v>-45.35794373959483</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3424200529802335</v>
+        <v>0.3424200529802336</v>
       </c>
       <c r="D6" t="n">
         <v>5.371792022318755</v>
       </c>
       <c r="E6" t="n">
-        <v>20.27325930605141</v>
+        <v>20.27325930605142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar pipeline, resultados y figuras de analisis geologico.
Sincroniza scripts de procesamiento/EDA/geostatistica junto con artefactos generados (tablas, predicciones e imagenes) para reflejar el estado local completo del proyecto.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/processed/Obs/metricas_ml_vs_kriging.xlsx
+++ b/data/processed/Obs/metricas_ml_vs_kriging.xlsx
@@ -538,16 +538,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-45.35794373959483</v>
+        <v>-45.35794373959484</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3424200529802336</v>
+        <v>0.3424200529802335</v>
       </c>
       <c r="D6" t="n">
         <v>5.371792022318755</v>
       </c>
       <c r="E6" t="n">
-        <v>20.27325930605142</v>
+        <v>20.27325930605141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>